<commit_message>
Update annex 11 to 87 samples and align annex descriptions with the thesis
</commit_message>
<xml_diff>
--- a/Anexo_11_Comparacion_articulo_guia/Anexo_11_Comparacion_articulo_guia.xlsx
+++ b/Anexo_11_Comparacion_articulo_guia/Anexo_11_Comparacion_articulo_guia.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>86/86 idénticas</t>
+          <t>87/87 idénticas</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.269 vs 0.679</t>
+          <t>0.269 vs 0.685</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>r = 0.9804</t>
+          <t>r = 0.9800</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>r = 0.9701</t>
+          <t>r = 0.9700</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>r = 0.9939, p = 0.001</t>
+          <t>r = 0.9940, p = 0.001</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O87"/>
+  <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -977,7 +977,7 @@
         <v>4.248569241955242</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2971553980309804</v>
+        <v>0.2971553980309803</v>
       </c>
     </row>
     <row r="6">
@@ -1091,7 +1091,7 @@
         <v>4.807469046789805</v>
       </c>
       <c r="O7" t="n">
-        <v>0.2891045978336745</v>
+        <v>0.2891045978336744</v>
       </c>
     </row>
     <row r="8">
@@ -1319,7 +1319,7 @@
         <v>4.621830396364131</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2755651951830796</v>
+        <v>0.2755651951830797</v>
       </c>
     </row>
     <row r="12">
@@ -1661,7 +1661,7 @@
         <v>5.188624611605985</v>
       </c>
       <c r="O17" t="n">
-        <v>0.241000749423276</v>
+        <v>0.2410007494232761</v>
       </c>
     </row>
     <row r="18">
@@ -1718,7 +1718,7 @@
         <v>5.257969617222424</v>
       </c>
       <c r="O18" t="n">
-        <v>0.2552545100978133</v>
+        <v>0.2552545100978134</v>
       </c>
     </row>
     <row r="19">
@@ -1769,7 +1769,7 @@
         <v>24721</v>
       </c>
       <c r="M19" t="n">
-        <v>5.002868496696968</v>
+        <v>5.00522300617649</v>
       </c>
       <c r="N19" t="n">
         <v>5.247143619338262</v>
@@ -2003,7 +2003,7 @@
         <v>4.532089573639797</v>
       </c>
       <c r="O23" t="n">
-        <v>0.2690354884567598</v>
+        <v>0.2690354884567599</v>
       </c>
     </row>
     <row r="24">
@@ -2060,7 +2060,7 @@
         <v>4.657884786275015</v>
       </c>
       <c r="O24" t="n">
-        <v>0.281549399569935</v>
+        <v>0.2815493995699349</v>
       </c>
     </row>
     <row r="25">
@@ -2174,7 +2174,7 @@
         <v>4.542889077396673</v>
       </c>
       <c r="O26" t="n">
-        <v>0.2800663229121658</v>
+        <v>0.2800663229121657</v>
       </c>
     </row>
     <row r="27">
@@ -2345,7 +2345,7 @@
         <v>4.663762916204359</v>
       </c>
       <c r="O29" t="n">
-        <v>0.2779152846712366</v>
+        <v>0.2779152846712367</v>
       </c>
     </row>
     <row r="30">
@@ -2453,7 +2453,7 @@
         <v>24505</v>
       </c>
       <c r="M31" t="n">
-        <v>4.86041379422328</v>
+        <v>4.862931335442059</v>
       </c>
       <c r="N31" t="n">
         <v>5.112906376202671</v>
@@ -2567,13 +2567,13 @@
         <v>32938</v>
       </c>
       <c r="M33" t="n">
-        <v>4.459702866895109</v>
+        <v>4.463773556967974</v>
       </c>
       <c r="N33" t="n">
         <v>4.786697684955428</v>
       </c>
       <c r="O33" t="n">
-        <v>0.2154323708791753</v>
+        <v>0.2154323708791752</v>
       </c>
     </row>
     <row r="34">
@@ -2915,7 +2915,7 @@
         <v>4.717655253883136</v>
       </c>
       <c r="O39" t="n">
-        <v>0.2840797004641687</v>
+        <v>0.2840797004641688</v>
       </c>
     </row>
     <row r="40">
@@ -3251,7 +3251,7 @@
         <v>13394</v>
       </c>
       <c r="M45" t="n">
-        <v>4.170742418295903</v>
+        <v>4.176448356873278</v>
       </c>
       <c r="N45" t="n">
         <v>4.57630739951137</v>
@@ -3314,7 +3314,7 @@
         <v>4.709457445226017</v>
       </c>
       <c r="O46" t="n">
-        <v>0.2309313957710923</v>
+        <v>0.2309313957710924</v>
       </c>
     </row>
     <row r="47">
@@ -3542,7 +3542,7 @@
         <v>4.59032512764368</v>
       </c>
       <c r="O50" t="n">
-        <v>0.268594637937662</v>
+        <v>0.2685946379376621</v>
       </c>
     </row>
     <row r="51">
@@ -4112,7 +4112,7 @@
         <v>4.487747967477103</v>
       </c>
       <c r="O60" t="n">
-        <v>0.2632830454531032</v>
+        <v>0.2632830454531033</v>
       </c>
     </row>
     <row r="61">
@@ -4226,7 +4226,7 @@
         <v>4.488940656499014</v>
       </c>
       <c r="O62" t="n">
-        <v>0.273775051455907</v>
+        <v>0.2737750514559069</v>
       </c>
     </row>
     <row r="63">
@@ -4397,7 +4397,7 @@
         <v>4.296682138811668</v>
       </c>
       <c r="O65" t="n">
-        <v>0.280419138078824</v>
+        <v>0.2804191380788239</v>
       </c>
     </row>
     <row r="66">
@@ -4511,7 +4511,7 @@
         <v>4.685229933478695</v>
       </c>
       <c r="O67" t="n">
-        <v>0.2747961933184367</v>
+        <v>0.2747961933184368</v>
       </c>
     </row>
     <row r="68">
@@ -4625,7 +4625,7 @@
         <v>5.040834697632513</v>
       </c>
       <c r="O69" t="n">
-        <v>0.2739443868143194</v>
+        <v>0.2739443868143195</v>
       </c>
     </row>
     <row r="70">
@@ -4967,7 +4967,7 @@
         <v>4.948808225371879</v>
       </c>
       <c r="O75" t="n">
-        <v>0.2710088589395876</v>
+        <v>0.2710088589395877</v>
       </c>
     </row>
     <row r="76">
@@ -5072,7 +5072,7 @@
         <v>21173</v>
       </c>
       <c r="L77" t="n">
-        <v>32543</v>
+        <v>32543.00000000001</v>
       </c>
       <c r="M77" t="n">
         <v>5.095258706793435</v>
@@ -5081,7 +5081,7 @@
         <v>5.24373219381151</v>
       </c>
       <c r="O77" t="n">
-        <v>0.2567669657322041</v>
+        <v>0.2567669657322042</v>
       </c>
     </row>
     <row r="78">
@@ -5252,7 +5252,7 @@
         <v>4.938340692114959</v>
       </c>
       <c r="O80" t="n">
-        <v>0.2368423677303974</v>
+        <v>0.2368423677303973</v>
       </c>
     </row>
     <row r="81">
@@ -5471,7 +5471,7 @@
         <v>9069</v>
       </c>
       <c r="L84" t="n">
-        <v>15910</v>
+        <v>15910.00000000001</v>
       </c>
       <c r="M84" t="n">
         <v>4.076046622495229</v>
@@ -5651,7 +5651,64 @@
         <v>4.796694279400795</v>
       </c>
       <c r="O87" t="n">
-        <v>0.2759835837192706</v>
+        <v>0.2759835837192705</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SRR26147494</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>S1A2_bac</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>barcode26</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>bag</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>CSSwP</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>43900163</v>
+      </c>
+      <c r="H88" t="n">
+        <v>43900163</v>
+      </c>
+      <c r="I88" t="n">
+        <v>30646</v>
+      </c>
+      <c r="J88" t="n">
+        <v>15742</v>
+      </c>
+      <c r="K88" t="n">
+        <v>14490</v>
+      </c>
+      <c r="L88" t="n">
+        <v>23377</v>
+      </c>
+      <c r="M88" t="n">
+        <v>4.422854536115111</v>
+      </c>
+      <c r="N88" t="n">
+        <v>4.742177999043804</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.2425458882024158</v>
       </c>
     </row>
   </sheetData>
@@ -5745,7 +5802,7 @@
         <v>0.195</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1397495797832498</v>
+        <v>0.1397051533152246</v>
       </c>
       <c r="G2" t="n">
         <v>0.452</v>
@@ -5776,10 +5833,10 @@
         <v>0.277</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1547220577804336</v>
+        <v>0.1547662422774261</v>
       </c>
       <c r="G3" t="n">
-        <v>0.217</v>
+        <v>0.19</v>
       </c>
       <c r="H3" t="n">
         <v>0.1716950342958104</v>
@@ -5807,7 +5864,7 @@
         <v>0.327</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1529570925432435</v>
+        <v>0.1529635995844162</v>
       </c>
       <c r="G4" t="n">
         <v>0.276</v>
@@ -5838,7 +5895,7 @@
         <v>0.037</v>
       </c>
       <c r="F5" t="n">
-        <v>0.156127234893206</v>
+        <v>0.156086185859524</v>
       </c>
       <c r="G5" t="n">
         <v>0.273</v>
@@ -5869,7 +5926,7 @@
         <v>0.328</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1492729110127897</v>
+        <v>0.1492621470310157</v>
       </c>
       <c r="G6" t="n">
         <v>0.37</v>
@@ -5900,7 +5957,7 @@
         <v>0.332</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1533426243897088</v>
+        <v>0.1533207659196227</v>
       </c>
       <c r="G7" t="n">
         <v>0.335</v>
@@ -5922,7 +5979,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
         <v>0.168807258</v>
@@ -5931,16 +5988,16 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2159567277160997</v>
+        <v>0.1771808056209678</v>
       </c>
       <c r="G8" t="n">
-        <v>0.315</v>
+        <v>0.288</v>
       </c>
       <c r="H8" t="n">
-        <v>0.207568214905908</v>
+        <v>0.161933697890416</v>
       </c>
       <c r="I8" t="n">
-        <v>0.422</v>
+        <v>0.398</v>
       </c>
     </row>
     <row r="9">
@@ -5962,7 +6019,7 @@
         <v>0.027</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1725642601467045</v>
+        <v>0.1724305916353526</v>
       </c>
       <c r="G9" t="n">
         <v>0.044</v>
@@ -5993,7 +6050,7 @@
         <v>0.022</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1868905499277201</v>
+        <v>0.1868802669000751</v>
       </c>
       <c r="G10" t="n">
         <v>0.028</v>
@@ -6024,7 +6081,7 @@
         <v>0.137</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1467147706526538</v>
+        <v>0.1466618366813701</v>
       </c>
       <c r="G11" t="n">
         <v>0.278</v>
@@ -6055,7 +6112,7 @@
         <v>0.025</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1954108539884605</v>
+        <v>0.1954454804302889</v>
       </c>
       <c r="G12" t="n">
         <v>0.028</v>

</xml_diff>

<commit_message>
Add per-sample Pearson and shared species to annex 11; link the pipeline branch
</commit_message>
<xml_diff>
--- a/Anexo_11_Comparacion_articulo_guia/Anexo_11_Comparacion_articulo_guia.xlsx
+++ b/Anexo_11_Comparacion_articulo_guia/Anexo_11_Comparacion_articulo_guia.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Por_muestra" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PERMANOVA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Medias_por_tipo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PERMANOVA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -562,83 +563,134 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6. Diversidad alfa</t>
+          <t>5. Composición</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Shannon por muestra (Pearson)</t>
+          <t>Pearson entre perfiles de la misma muestra (mediana, mín–máx)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>r = 0.9800</t>
+          <t>r = 0.959 (0.854–0.978)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6. Diversidad alfa</t>
+          <t>5. Composición</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Riqueza observada por muestra (Pearson)</t>
+          <t>Especies compartidas por muestra (mediana)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>r = 0.9700</t>
+          <t>172 de 350 (48.9 %)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7. Diversidad beta</t>
+          <t>5. Composición</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mantel, distancias de Aitchison</t>
+          <t>Lecturas en especies compartidas (mediana)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>r = 0.9940, p = 0.001</t>
+          <t>este trabajo 93.1 %; artículo 82.1 %</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7. Diversidad beta</t>
+          <t>6. Diversidad alfa</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mantel, distancias de Bray-Curtis</t>
+          <t>Shannon por muestra (Pearson)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>r = 0.9990, p = 0.001</t>
+          <t>r = 0.9800</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>6. Diversidad alfa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Riqueza observada por muestra (Pearson)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>r = 0.9700</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7. Diversidad beta</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mantel, distancias de Aitchison</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>r = 0.9940, p = 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>7. Diversidad beta</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mantel, distancias de Bray-Curtis</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>r = 0.9990, p = 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>8. PERMANOVA</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Subconjuntos con la misma conclusión (α = 0.05)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>10 de 11</t>
         </is>
@@ -655,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O88"/>
+  <dimension ref="A1:W88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -672,7 +724,15 @@
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="31" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="22" max="22"/>
+    <col width="38" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -748,7 +808,47 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>Riqueza (este trabajo)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Riqueza (artículo)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Bray-Curtis misma muestra</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Pearson misma muestra</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Especies compartidas</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Especies solo en este trabajo</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Especies solo en el artículo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>% lecturas en compartidas (este trabajo)</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>% lecturas en compartidas (artículo)</t>
         </is>
       </c>
     </row>
@@ -806,7 +906,31 @@
         <v>4.915611415986612</v>
       </c>
       <c r="O2" t="n">
+        <v>226</v>
+      </c>
+      <c r="P2" t="n">
+        <v>326</v>
+      </c>
+      <c r="Q2" t="n">
         <v>0.2463366125597615</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.9386492978598479</v>
+      </c>
+      <c r="S2" t="n">
+        <v>209</v>
+      </c>
+      <c r="T2" t="n">
+        <v>24</v>
+      </c>
+      <c r="U2" t="n">
+        <v>123</v>
+      </c>
+      <c r="V2" t="n">
+        <v>96.09804197774335</v>
+      </c>
+      <c r="W2" t="n">
+        <v>87.31965954808626</v>
       </c>
     </row>
     <row r="3">
@@ -863,7 +987,31 @@
         <v>4.650643967856745</v>
       </c>
       <c r="O3" t="n">
+        <v>203</v>
+      </c>
+      <c r="P3" t="n">
+        <v>318</v>
+      </c>
+      <c r="Q3" t="n">
         <v>0.2726579185708702</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.9778577911643594</v>
+      </c>
+      <c r="S3" t="n">
+        <v>169</v>
+      </c>
+      <c r="T3" t="n">
+        <v>34</v>
+      </c>
+      <c r="U3" t="n">
+        <v>180</v>
+      </c>
+      <c r="V3" t="n">
+        <v>93.28025003720791</v>
+      </c>
+      <c r="W3" t="n">
+        <v>80.3671587133688</v>
       </c>
     </row>
     <row r="4">
@@ -920,7 +1068,31 @@
         <v>4.523464831448581</v>
       </c>
       <c r="O4" t="n">
+        <v>158</v>
+      </c>
+      <c r="P4" t="n">
+        <v>246</v>
+      </c>
+      <c r="Q4" t="n">
         <v>0.2727206456136145</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.9704538877289696</v>
+      </c>
+      <c r="S4" t="n">
+        <v>133</v>
+      </c>
+      <c r="T4" t="n">
+        <v>25</v>
+      </c>
+      <c r="U4" t="n">
+        <v>138</v>
+      </c>
+      <c r="V4" t="n">
+        <v>93.09815950920246</v>
+      </c>
+      <c r="W4" t="n">
+        <v>78.75445760245705</v>
       </c>
     </row>
     <row r="5">
@@ -977,7 +1149,31 @@
         <v>4.248569241955242</v>
       </c>
       <c r="O5" t="n">
+        <v>112</v>
+      </c>
+      <c r="P5" t="n">
+        <v>174</v>
+      </c>
+      <c r="Q5" t="n">
         <v>0.2971553980309803</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.9594104203434275</v>
+      </c>
+      <c r="S5" t="n">
+        <v>88</v>
+      </c>
+      <c r="T5" t="n">
+        <v>24</v>
+      </c>
+      <c r="U5" t="n">
+        <v>106</v>
+      </c>
+      <c r="V5" t="n">
+        <v>89.66555714059281</v>
+      </c>
+      <c r="W5" t="n">
+        <v>77.59196538126858</v>
       </c>
     </row>
     <row r="6">
@@ -1034,7 +1230,31 @@
         <v>4.837683567164206</v>
       </c>
       <c r="O6" t="n">
+        <v>254</v>
+      </c>
+      <c r="P6" t="n">
+        <v>358</v>
+      </c>
+      <c r="Q6" t="n">
         <v>0.2714388021087945</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.965577249353672</v>
+      </c>
+      <c r="S6" t="n">
+        <v>211</v>
+      </c>
+      <c r="T6" t="n">
+        <v>49</v>
+      </c>
+      <c r="U6" t="n">
+        <v>181</v>
+      </c>
+      <c r="V6" t="n">
+        <v>92.49697702539299</v>
+      </c>
+      <c r="W6" t="n">
+        <v>83.21711849001383</v>
       </c>
     </row>
     <row r="7">
@@ -1091,7 +1311,31 @@
         <v>4.807469046789805</v>
       </c>
       <c r="O7" t="n">
+        <v>214</v>
+      </c>
+      <c r="P7" t="n">
+        <v>311</v>
+      </c>
+      <c r="Q7" t="n">
         <v>0.2891045978336744</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.9502436603397143</v>
+      </c>
+      <c r="S7" t="n">
+        <v>181</v>
+      </c>
+      <c r="T7" t="n">
+        <v>38</v>
+      </c>
+      <c r="U7" t="n">
+        <v>166</v>
+      </c>
+      <c r="V7" t="n">
+        <v>92.65426815033851</v>
+      </c>
+      <c r="W7" t="n">
+        <v>80.64581716408003</v>
       </c>
     </row>
     <row r="8">
@@ -1148,7 +1392,31 @@
         <v>4.742150854054434</v>
       </c>
       <c r="O8" t="n">
+        <v>209</v>
+      </c>
+      <c r="P8" t="n">
+        <v>316</v>
+      </c>
+      <c r="Q8" t="n">
         <v>0.2797162712371907</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.9548889942568927</v>
+      </c>
+      <c r="S8" t="n">
+        <v>184</v>
+      </c>
+      <c r="T8" t="n">
+        <v>33</v>
+      </c>
+      <c r="U8" t="n">
+        <v>165</v>
+      </c>
+      <c r="V8" t="n">
+        <v>93.26746166950596</v>
+      </c>
+      <c r="W8" t="n">
+        <v>81.56302997355706</v>
       </c>
     </row>
     <row r="9">
@@ -1205,7 +1473,31 @@
         <v>4.85252723432548</v>
       </c>
       <c r="O9" t="n">
+        <v>248</v>
+      </c>
+      <c r="P9" t="n">
+        <v>363</v>
+      </c>
+      <c r="Q9" t="n">
         <v>0.2680679218831823</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.9695202276819344</v>
+      </c>
+      <c r="S9" t="n">
+        <v>220</v>
+      </c>
+      <c r="T9" t="n">
+        <v>32</v>
+      </c>
+      <c r="U9" t="n">
+        <v>179</v>
+      </c>
+      <c r="V9" t="n">
+        <v>94.74343712799951</v>
+      </c>
+      <c r="W9" t="n">
+        <v>82.7085370898353</v>
       </c>
     </row>
     <row r="10">
@@ -1262,7 +1554,31 @@
         <v>4.931017839487023</v>
       </c>
       <c r="O10" t="n">
+        <v>257</v>
+      </c>
+      <c r="P10" t="n">
+        <v>407</v>
+      </c>
+      <c r="Q10" t="n">
         <v>0.271821401222459</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.9677862370540289</v>
+      </c>
+      <c r="S10" t="n">
+        <v>230</v>
+      </c>
+      <c r="T10" t="n">
+        <v>36</v>
+      </c>
+      <c r="U10" t="n">
+        <v>215</v>
+      </c>
+      <c r="V10" t="n">
+        <v>94.43853427895981</v>
+      </c>
+      <c r="W10" t="n">
+        <v>81.22935042075945</v>
       </c>
     </row>
     <row r="11">
@@ -1319,7 +1635,31 @@
         <v>4.621830396364131</v>
       </c>
       <c r="O11" t="n">
+        <v>222</v>
+      </c>
+      <c r="P11" t="n">
+        <v>319</v>
+      </c>
+      <c r="Q11" t="n">
         <v>0.2755651951830797</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.9678083193797092</v>
+      </c>
+      <c r="S11" t="n">
+        <v>184</v>
+      </c>
+      <c r="T11" t="n">
+        <v>40</v>
+      </c>
+      <c r="U11" t="n">
+        <v>172</v>
+      </c>
+      <c r="V11" t="n">
+        <v>93.30339453176595</v>
+      </c>
+      <c r="W11" t="n">
+        <v>81.67011598928188</v>
       </c>
     </row>
     <row r="12">
@@ -1376,7 +1716,31 @@
         <v>5.141000587414185</v>
       </c>
       <c r="O12" t="n">
+        <v>263</v>
+      </c>
+      <c r="P12" t="n">
+        <v>354</v>
+      </c>
+      <c r="Q12" t="n">
         <v>0.2584861562334144</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.9220646727392386</v>
+      </c>
+      <c r="S12" t="n">
+        <v>228</v>
+      </c>
+      <c r="T12" t="n">
+        <v>42</v>
+      </c>
+      <c r="U12" t="n">
+        <v>136</v>
+      </c>
+      <c r="V12" t="n">
+        <v>94.23424676589235</v>
+      </c>
+      <c r="W12" t="n">
+        <v>86.15879833468385</v>
       </c>
     </row>
     <row r="13">
@@ -1433,7 +1797,31 @@
         <v>4.562010657832851</v>
       </c>
       <c r="O13" t="n">
+        <v>178</v>
+      </c>
+      <c r="P13" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q13" t="n">
         <v>0.2621916720204812</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.9679277179368717</v>
+      </c>
+      <c r="S13" t="n">
+        <v>153</v>
+      </c>
+      <c r="T13" t="n">
+        <v>27</v>
+      </c>
+      <c r="U13" t="n">
+        <v>126</v>
+      </c>
+      <c r="V13" t="n">
+        <v>93.37249143416544</v>
+      </c>
+      <c r="W13" t="n">
+        <v>81.38063709340749</v>
       </c>
     </row>
     <row r="14">
@@ -1490,7 +1878,31 @@
         <v>4.890591407061016</v>
       </c>
       <c r="O14" t="n">
+        <v>188</v>
+      </c>
+      <c r="P14" t="n">
+        <v>244</v>
+      </c>
+      <c r="Q14" t="n">
         <v>0.2412492633187513</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.9325292145221349</v>
+      </c>
+      <c r="S14" t="n">
+        <v>160</v>
+      </c>
+      <c r="T14" t="n">
+        <v>29</v>
+      </c>
+      <c r="U14" t="n">
+        <v>94</v>
+      </c>
+      <c r="V14" t="n">
+        <v>91.86608122941824</v>
+      </c>
+      <c r="W14" t="n">
+        <v>85.79826239918134</v>
       </c>
     </row>
     <row r="15">
@@ -1547,7 +1959,31 @@
         <v>5.008945936460351</v>
       </c>
       <c r="O15" t="n">
+        <v>217</v>
+      </c>
+      <c r="P15" t="n">
+        <v>315</v>
+      </c>
+      <c r="Q15" t="n">
         <v>0.2519097062865474</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.9436152667980815</v>
+      </c>
+      <c r="S15" t="n">
+        <v>199</v>
+      </c>
+      <c r="T15" t="n">
+        <v>21</v>
+      </c>
+      <c r="U15" t="n">
+        <v>131</v>
+      </c>
+      <c r="V15" t="n">
+        <v>96.41135088135326</v>
+      </c>
+      <c r="W15" t="n">
+        <v>84.22502891070816</v>
       </c>
     </row>
     <row r="16">
@@ -1604,7 +2040,31 @@
         <v>5.1348790580715</v>
       </c>
       <c r="O16" t="n">
+        <v>234</v>
+      </c>
+      <c r="P16" t="n">
+        <v>327</v>
+      </c>
+      <c r="Q16" t="n">
         <v>0.2556795495968582</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.9122408013625137</v>
+      </c>
+      <c r="S16" t="n">
+        <v>202</v>
+      </c>
+      <c r="T16" t="n">
+        <v>32</v>
+      </c>
+      <c r="U16" t="n">
+        <v>135</v>
+      </c>
+      <c r="V16" t="n">
+        <v>93.68060091443499</v>
+      </c>
+      <c r="W16" t="n">
+        <v>84.01530251373323</v>
       </c>
     </row>
     <row r="17">
@@ -1661,7 +2121,31 @@
         <v>5.188624611605985</v>
       </c>
       <c r="O17" t="n">
+        <v>240</v>
+      </c>
+      <c r="P17" t="n">
+        <v>341</v>
+      </c>
+      <c r="Q17" t="n">
         <v>0.2410007494232761</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0.9325607021603622</v>
+      </c>
+      <c r="S17" t="n">
+        <v>214</v>
+      </c>
+      <c r="T17" t="n">
+        <v>26</v>
+      </c>
+      <c r="U17" t="n">
+        <v>139</v>
+      </c>
+      <c r="V17" t="n">
+        <v>95.13945402086262</v>
+      </c>
+      <c r="W17" t="n">
+        <v>84.70135957653257</v>
       </c>
     </row>
     <row r="18">
@@ -1718,7 +2202,31 @@
         <v>5.257969617222424</v>
       </c>
       <c r="O18" t="n">
+        <v>272</v>
+      </c>
+      <c r="P18" t="n">
+        <v>355</v>
+      </c>
+      <c r="Q18" t="n">
         <v>0.2552545100978134</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.8886204496511051</v>
+      </c>
+      <c r="S18" t="n">
+        <v>234</v>
+      </c>
+      <c r="T18" t="n">
+        <v>43</v>
+      </c>
+      <c r="U18" t="n">
+        <v>133</v>
+      </c>
+      <c r="V18" t="n">
+        <v>94.20150788211103</v>
+      </c>
+      <c r="W18" t="n">
+        <v>86.00979206252867</v>
       </c>
     </row>
     <row r="19">
@@ -1775,7 +2283,31 @@
         <v>5.247143619338262</v>
       </c>
       <c r="O19" t="n">
+        <v>252</v>
+      </c>
+      <c r="P19" t="n">
+        <v>364</v>
+      </c>
+      <c r="Q19" t="n">
         <v>0.2465088685504498</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.9082210208486398</v>
+      </c>
+      <c r="S19" t="n">
+        <v>228</v>
+      </c>
+      <c r="T19" t="n">
+        <v>30</v>
+      </c>
+      <c r="U19" t="n">
+        <v>152</v>
+      </c>
+      <c r="V19" t="n">
+        <v>94.97557110788327</v>
+      </c>
+      <c r="W19" t="n">
+        <v>84.92637570511732</v>
       </c>
     </row>
     <row r="20">
@@ -1832,7 +2364,31 @@
         <v>4.99473753851898</v>
       </c>
       <c r="O20" t="n">
+        <v>237</v>
+      </c>
+      <c r="P20" t="n">
+        <v>335</v>
+      </c>
+      <c r="Q20" t="n">
         <v>0.2483488235623901</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.9391470679121529</v>
+      </c>
+      <c r="S20" t="n">
+        <v>203</v>
+      </c>
+      <c r="T20" t="n">
+        <v>36</v>
+      </c>
+      <c r="U20" t="n">
+        <v>142</v>
+      </c>
+      <c r="V20" t="n">
+        <v>94.48025233132201</v>
+      </c>
+      <c r="W20" t="n">
+        <v>85.97519934051749</v>
       </c>
     </row>
     <row r="21">
@@ -1889,7 +2445,31 @@
         <v>4.905242813813881</v>
       </c>
       <c r="O21" t="n">
+        <v>271</v>
+      </c>
+      <c r="P21" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q21" t="n">
         <v>0.2740679411248794</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.9688651513856259</v>
+      </c>
+      <c r="S21" t="n">
+        <v>232</v>
+      </c>
+      <c r="T21" t="n">
+        <v>51</v>
+      </c>
+      <c r="U21" t="n">
+        <v>203</v>
+      </c>
+      <c r="V21" t="n">
+        <v>92.42543376841222</v>
+      </c>
+      <c r="W21" t="n">
+        <v>82.68699168076529</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +2526,31 @@
         <v>4.285110195847912</v>
       </c>
       <c r="O22" t="n">
+        <v>129</v>
+      </c>
+      <c r="P22" t="n">
+        <v>204</v>
+      </c>
+      <c r="Q22" t="n">
         <v>0.2688710543699575</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.9710603809398239</v>
+      </c>
+      <c r="S22" t="n">
+        <v>114</v>
+      </c>
+      <c r="T22" t="n">
+        <v>17</v>
+      </c>
+      <c r="U22" t="n">
+        <v>112</v>
+      </c>
+      <c r="V22" t="n">
+        <v>94.08765327182226</v>
+      </c>
+      <c r="W22" t="n">
+        <v>80.03763276963039</v>
       </c>
     </row>
     <row r="23">
@@ -2003,7 +2607,31 @@
         <v>4.532089573639797</v>
       </c>
       <c r="O23" t="n">
+        <v>177</v>
+      </c>
+      <c r="P23" t="n">
+        <v>243</v>
+      </c>
+      <c r="Q23" t="n">
         <v>0.2690354884567599</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.9650516567729238</v>
+      </c>
+      <c r="S23" t="n">
+        <v>148</v>
+      </c>
+      <c r="T23" t="n">
+        <v>31</v>
+      </c>
+      <c r="U23" t="n">
+        <v>126</v>
+      </c>
+      <c r="V23" t="n">
+        <v>92.36648424230987</v>
+      </c>
+      <c r="W23" t="n">
+        <v>82.12213165121008</v>
       </c>
     </row>
     <row r="24">
@@ -2060,7 +2688,31 @@
         <v>4.657884786275015</v>
       </c>
       <c r="O24" t="n">
+        <v>201</v>
+      </c>
+      <c r="P24" t="n">
+        <v>312</v>
+      </c>
+      <c r="Q24" t="n">
         <v>0.2815493995699349</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.9655739447247551</v>
+      </c>
+      <c r="S24" t="n">
+        <v>172</v>
+      </c>
+      <c r="T24" t="n">
+        <v>29</v>
+      </c>
+      <c r="U24" t="n">
+        <v>178</v>
+      </c>
+      <c r="V24" t="n">
+        <v>93.80727165237954</v>
+      </c>
+      <c r="W24" t="n">
+        <v>79.68329104697183</v>
       </c>
     </row>
     <row r="25">
@@ -2117,7 +2769,31 @@
         <v>5.064370885317422</v>
       </c>
       <c r="O25" t="n">
+        <v>285</v>
+      </c>
+      <c r="P25" t="n">
+        <v>420</v>
+      </c>
+      <c r="Q25" t="n">
         <v>0.2827814473652545</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0.9510971758378574</v>
+      </c>
+      <c r="S25" t="n">
+        <v>245</v>
+      </c>
+      <c r="T25" t="n">
+        <v>44</v>
+      </c>
+      <c r="U25" t="n">
+        <v>218</v>
+      </c>
+      <c r="V25" t="n">
+        <v>93.5035445281347</v>
+      </c>
+      <c r="W25" t="n">
+        <v>82.64594952951259</v>
       </c>
     </row>
     <row r="26">
@@ -2174,7 +2850,31 @@
         <v>4.542889077396673</v>
       </c>
       <c r="O26" t="n">
+        <v>178</v>
+      </c>
+      <c r="P26" t="n">
+        <v>259</v>
+      </c>
+      <c r="Q26" t="n">
         <v>0.2800663229121657</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.9648009377538697</v>
+      </c>
+      <c r="S26" t="n">
+        <v>144</v>
+      </c>
+      <c r="T26" t="n">
+        <v>35</v>
+      </c>
+      <c r="U26" t="n">
+        <v>145</v>
+      </c>
+      <c r="V26" t="n">
+        <v>91.3522717089345</v>
+      </c>
+      <c r="W26" t="n">
+        <v>80.80991149480906</v>
       </c>
     </row>
     <row r="27">
@@ -2231,7 +2931,31 @@
         <v>4.308792281101613</v>
       </c>
       <c r="O27" t="n">
+        <v>134</v>
+      </c>
+      <c r="P27" t="n">
+        <v>188</v>
+      </c>
+      <c r="Q27" t="n">
         <v>0.2681153098636731</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0.9665828881152796</v>
+      </c>
+      <c r="S27" t="n">
+        <v>114</v>
+      </c>
+      <c r="T27" t="n">
+        <v>20</v>
+      </c>
+      <c r="U27" t="n">
+        <v>96</v>
+      </c>
+      <c r="V27" t="n">
+        <v>92.02388852023888</v>
+      </c>
+      <c r="W27" t="n">
+        <v>81.83638077025702</v>
       </c>
     </row>
     <row r="28">
@@ -2288,7 +3012,31 @@
         <v>5.030181691911634</v>
       </c>
       <c r="O28" t="n">
+        <v>221</v>
+      </c>
+      <c r="P28" t="n">
+        <v>307</v>
+      </c>
+      <c r="Q28" t="n">
         <v>0.2400232951756898</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0.9418806797641396</v>
+      </c>
+      <c r="S28" t="n">
+        <v>192</v>
+      </c>
+      <c r="T28" t="n">
+        <v>31</v>
+      </c>
+      <c r="U28" t="n">
+        <v>127</v>
+      </c>
+      <c r="V28" t="n">
+        <v>94.68757135246213</v>
+      </c>
+      <c r="W28" t="n">
+        <v>85.32974217229996</v>
       </c>
     </row>
     <row r="29">
@@ -2345,7 +3093,31 @@
         <v>4.663762916204359</v>
       </c>
       <c r="O29" t="n">
+        <v>196</v>
+      </c>
+      <c r="P29" t="n">
+        <v>288</v>
+      </c>
+      <c r="Q29" t="n">
         <v>0.2779152846712367</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.965076896999694</v>
+      </c>
+      <c r="S29" t="n">
+        <v>166</v>
+      </c>
+      <c r="T29" t="n">
+        <v>32</v>
+      </c>
+      <c r="U29" t="n">
+        <v>152</v>
+      </c>
+      <c r="V29" t="n">
+        <v>92.62769437222177</v>
+      </c>
+      <c r="W29" t="n">
+        <v>81.31350458797073</v>
       </c>
     </row>
     <row r="30">
@@ -2402,7 +3174,31 @@
         <v>5.119778872160603</v>
       </c>
       <c r="O30" t="n">
+        <v>240</v>
+      </c>
+      <c r="P30" t="n">
+        <v>319</v>
+      </c>
+      <c r="Q30" t="n">
         <v>0.2359173211970825</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0.9384640497119042</v>
+      </c>
+      <c r="S30" t="n">
+        <v>219</v>
+      </c>
+      <c r="T30" t="n">
+        <v>29</v>
+      </c>
+      <c r="U30" t="n">
+        <v>116</v>
+      </c>
+      <c r="V30" t="n">
+        <v>95.45268052516411</v>
+      </c>
+      <c r="W30" t="n">
+        <v>87.60468079499068</v>
       </c>
     </row>
     <row r="31">
@@ -2459,7 +3255,31 @@
         <v>5.112906376202671</v>
       </c>
       <c r="O31" t="n">
+        <v>237</v>
+      </c>
+      <c r="P31" t="n">
+        <v>351</v>
+      </c>
+      <c r="Q31" t="n">
         <v>0.2386962632997243</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.935425946550796</v>
+      </c>
+      <c r="S31" t="n">
+        <v>220</v>
+      </c>
+      <c r="T31" t="n">
+        <v>22</v>
+      </c>
+      <c r="U31" t="n">
+        <v>141</v>
+      </c>
+      <c r="V31" t="n">
+        <v>96.69172932330827</v>
+      </c>
+      <c r="W31" t="n">
+        <v>86.1162481064496</v>
       </c>
     </row>
     <row r="32">
@@ -2516,7 +3336,31 @@
         <v>4.569086723302096</v>
       </c>
       <c r="O32" t="n">
+        <v>141</v>
+      </c>
+      <c r="P32" t="n">
+        <v>224</v>
+      </c>
+      <c r="Q32" t="n">
         <v>0.2363973713868683</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0.9462927353371104</v>
+      </c>
+      <c r="S32" t="n">
+        <v>136</v>
+      </c>
+      <c r="T32" t="n">
+        <v>17</v>
+      </c>
+      <c r="U32" t="n">
+        <v>97</v>
+      </c>
+      <c r="V32" t="n">
+        <v>96.54132314498291</v>
+      </c>
+      <c r="W32" t="n">
+        <v>83.03367416707962</v>
       </c>
     </row>
     <row r="33">
@@ -2573,7 +3417,31 @@
         <v>4.786697684955428</v>
       </c>
       <c r="O33" t="n">
+        <v>225</v>
+      </c>
+      <c r="P33" t="n">
+        <v>355</v>
+      </c>
+      <c r="Q33" t="n">
         <v>0.2154323708791752</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.9711285085977341</v>
+      </c>
+      <c r="S33" t="n">
+        <v>226</v>
+      </c>
+      <c r="T33" t="n">
+        <v>20</v>
+      </c>
+      <c r="U33" t="n">
+        <v>144</v>
+      </c>
+      <c r="V33" t="n">
+        <v>97.57185332011893</v>
+      </c>
+      <c r="W33" t="n">
+        <v>88.71456621889836</v>
       </c>
     </row>
     <row r="34">
@@ -2630,7 +3498,31 @@
         <v>4.013534589398891</v>
       </c>
       <c r="O34" t="n">
+        <v>98</v>
+      </c>
+      <c r="P34" t="n">
+        <v>146</v>
+      </c>
+      <c r="Q34" t="n">
         <v>0.2540064193547975</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.9743417143341148</v>
+      </c>
+      <c r="S34" t="n">
+        <v>78</v>
+      </c>
+      <c r="T34" t="n">
+        <v>20</v>
+      </c>
+      <c r="U34" t="n">
+        <v>78</v>
+      </c>
+      <c r="V34" t="n">
+        <v>90.94650205761317</v>
+      </c>
+      <c r="W34" t="n">
+        <v>79.95458246890948</v>
       </c>
     </row>
     <row r="35">
@@ -2687,7 +3579,31 @@
         <v>4.481062033976776</v>
       </c>
       <c r="O35" t="n">
+        <v>153</v>
+      </c>
+      <c r="P35" t="n">
+        <v>227</v>
+      </c>
+      <c r="Q35" t="n">
         <v>0.2792300960676979</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0.9657288155809721</v>
+      </c>
+      <c r="S35" t="n">
+        <v>132</v>
+      </c>
+      <c r="T35" t="n">
+        <v>26</v>
+      </c>
+      <c r="U35" t="n">
+        <v>125</v>
+      </c>
+      <c r="V35" t="n">
+        <v>92.54162812210916</v>
+      </c>
+      <c r="W35" t="n">
+        <v>79.2358395980315</v>
       </c>
     </row>
     <row r="36">
@@ -2744,7 +3660,31 @@
         <v>4.643995235243666</v>
       </c>
       <c r="O36" t="n">
+        <v>199</v>
+      </c>
+      <c r="P36" t="n">
+        <v>290</v>
+      </c>
+      <c r="Q36" t="n">
         <v>0.2742914127031163</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0.9645591033287007</v>
+      </c>
+      <c r="S36" t="n">
+        <v>169</v>
+      </c>
+      <c r="T36" t="n">
+        <v>32</v>
+      </c>
+      <c r="U36" t="n">
+        <v>154</v>
+      </c>
+      <c r="V36" t="n">
+        <v>93.32637327336974</v>
+      </c>
+      <c r="W36" t="n">
+        <v>80.55183007101743</v>
       </c>
     </row>
     <row r="37">
@@ -2801,7 +3741,31 @@
         <v>4.794469195486333</v>
       </c>
       <c r="O37" t="n">
+        <v>256</v>
+      </c>
+      <c r="P37" t="n">
+        <v>350</v>
+      </c>
+      <c r="Q37" t="n">
         <v>0.2779546200255714</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0.9689213195433051</v>
+      </c>
+      <c r="S37" t="n">
+        <v>199</v>
+      </c>
+      <c r="T37" t="n">
+        <v>58</v>
+      </c>
+      <c r="U37" t="n">
+        <v>189</v>
+      </c>
+      <c r="V37" t="n">
+        <v>90.85255892046513</v>
+      </c>
+      <c r="W37" t="n">
+        <v>81.83199667837933</v>
       </c>
     </row>
     <row r="38">
@@ -2858,7 +3822,31 @@
         <v>4.556257528993052</v>
       </c>
       <c r="O38" t="n">
+        <v>152</v>
+      </c>
+      <c r="P38" t="n">
+        <v>252</v>
+      </c>
+      <c r="Q38" t="n">
         <v>0.2890503602646195</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.96152477325095</v>
+      </c>
+      <c r="S38" t="n">
+        <v>130</v>
+      </c>
+      <c r="T38" t="n">
+        <v>22</v>
+      </c>
+      <c r="U38" t="n">
+        <v>148</v>
+      </c>
+      <c r="V38" t="n">
+        <v>93.52935191779427</v>
+      </c>
+      <c r="W38" t="n">
+        <v>77.49873466095517</v>
       </c>
     </row>
     <row r="39">
@@ -2915,7 +3903,31 @@
         <v>4.717655253883136</v>
       </c>
       <c r="O39" t="n">
+        <v>215</v>
+      </c>
+      <c r="P39" t="n">
+        <v>316</v>
+      </c>
+      <c r="Q39" t="n">
         <v>0.2840797004641688</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.9653528621411039</v>
+      </c>
+      <c r="S39" t="n">
+        <v>178</v>
+      </c>
+      <c r="T39" t="n">
+        <v>38</v>
+      </c>
+      <c r="U39" t="n">
+        <v>174</v>
+      </c>
+      <c r="V39" t="n">
+        <v>92.38445378151259</v>
+      </c>
+      <c r="W39" t="n">
+        <v>80.21043829889865</v>
       </c>
     </row>
     <row r="40">
@@ -2972,7 +3984,31 @@
         <v>4.180647802566308</v>
       </c>
       <c r="O40" t="n">
+        <v>112</v>
+      </c>
+      <c r="P40" t="n">
+        <v>181</v>
+      </c>
+      <c r="Q40" t="n">
         <v>0.2697915315439438</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0.9731091242414249</v>
+      </c>
+      <c r="S40" t="n">
+        <v>92</v>
+      </c>
+      <c r="T40" t="n">
+        <v>20</v>
+      </c>
+      <c r="U40" t="n">
+        <v>106</v>
+      </c>
+      <c r="V40" t="n">
+        <v>92.20926926357691</v>
+      </c>
+      <c r="W40" t="n">
+        <v>79.39547359249268</v>
       </c>
     </row>
     <row r="41">
@@ -3029,7 +4065,31 @@
         <v>4.979173198317154</v>
       </c>
       <c r="O41" t="n">
+        <v>272</v>
+      </c>
+      <c r="P41" t="n">
+        <v>381</v>
+      </c>
+      <c r="Q41" t="n">
         <v>0.2458304098134624</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0.9525246543680699</v>
+      </c>
+      <c r="S41" t="n">
+        <v>241</v>
+      </c>
+      <c r="T41" t="n">
+        <v>38</v>
+      </c>
+      <c r="U41" t="n">
+        <v>152</v>
+      </c>
+      <c r="V41" t="n">
+        <v>95.70936091222488</v>
+      </c>
+      <c r="W41" t="n">
+        <v>87.82510035525344</v>
       </c>
     </row>
     <row r="42">
@@ -3086,7 +4146,31 @@
         <v>4.435330583569984</v>
       </c>
       <c r="O42" t="n">
+        <v>143</v>
+      </c>
+      <c r="P42" t="n">
+        <v>199</v>
+      </c>
+      <c r="Q42" t="n">
         <v>0.2878454114712858</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0.9469637132742167</v>
+      </c>
+      <c r="S42" t="n">
+        <v>117</v>
+      </c>
+      <c r="T42" t="n">
+        <v>26</v>
+      </c>
+      <c r="U42" t="n">
+        <v>113</v>
+      </c>
+      <c r="V42" t="n">
+        <v>91.13236814891415</v>
+      </c>
+      <c r="W42" t="n">
+        <v>80.78007184877374</v>
       </c>
     </row>
     <row r="43">
@@ -3143,7 +4227,31 @@
         <v>5.058490468733408</v>
       </c>
       <c r="O43" t="n">
+        <v>303</v>
+      </c>
+      <c r="P43" t="n">
+        <v>443</v>
+      </c>
+      <c r="Q43" t="n">
         <v>0.2799881202566968</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0.9606453198148104</v>
+      </c>
+      <c r="S43" t="n">
+        <v>259</v>
+      </c>
+      <c r="T43" t="n">
+        <v>60</v>
+      </c>
+      <c r="U43" t="n">
+        <v>225</v>
+      </c>
+      <c r="V43" t="n">
+        <v>92.32489933886761</v>
+      </c>
+      <c r="W43" t="n">
+        <v>82.68264060264649</v>
       </c>
     </row>
     <row r="44">
@@ -3200,7 +4308,31 @@
         <v>4.696459189700441</v>
       </c>
       <c r="O44" t="n">
+        <v>193</v>
+      </c>
+      <c r="P44" t="n">
+        <v>292</v>
+      </c>
+      <c r="Q44" t="n">
         <v>0.2776908383946394</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0.9682716266632618</v>
+      </c>
+      <c r="S44" t="n">
+        <v>164</v>
+      </c>
+      <c r="T44" t="n">
+        <v>32</v>
+      </c>
+      <c r="U44" t="n">
+        <v>157</v>
+      </c>
+      <c r="V44" t="n">
+        <v>93.07916881332648</v>
+      </c>
+      <c r="W44" t="n">
+        <v>80.06430445135624</v>
       </c>
     </row>
     <row r="45">
@@ -3257,7 +4389,31 @@
         <v>4.57630739951137</v>
       </c>
       <c r="O45" t="n">
+        <v>117</v>
+      </c>
+      <c r="P45" t="n">
+        <v>185</v>
+      </c>
+      <c r="Q45" t="n">
         <v>0.252067417316353</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0.9277442845352262</v>
+      </c>
+      <c r="S45" t="n">
+        <v>110</v>
+      </c>
+      <c r="T45" t="n">
+        <v>12</v>
+      </c>
+      <c r="U45" t="n">
+        <v>81</v>
+      </c>
+      <c r="V45" t="n">
+        <v>96.44187008688456</v>
+      </c>
+      <c r="W45" t="n">
+        <v>81.73050444087022</v>
       </c>
     </row>
     <row r="46">
@@ -3314,7 +4470,31 @@
         <v>4.709457445226017</v>
       </c>
       <c r="O46" t="n">
+        <v>224</v>
+      </c>
+      <c r="P46" t="n">
+        <v>343</v>
+      </c>
+      <c r="Q46" t="n">
         <v>0.2309313957710924</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0.9511061802293161</v>
+      </c>
+      <c r="S46" t="n">
+        <v>208</v>
+      </c>
+      <c r="T46" t="n">
+        <v>27</v>
+      </c>
+      <c r="U46" t="n">
+        <v>141</v>
+      </c>
+      <c r="V46" t="n">
+        <v>97.04400915797507</v>
+      </c>
+      <c r="W46" t="n">
+        <v>88.30136644687838</v>
       </c>
     </row>
     <row r="47">
@@ -3371,7 +4551,31 @@
         <v>4.872491848988113</v>
       </c>
       <c r="O47" t="n">
+        <v>259</v>
+      </c>
+      <c r="P47" t="n">
+        <v>403</v>
+      </c>
+      <c r="Q47" t="n">
         <v>0.2708420256800295</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.9653247125498586</v>
+      </c>
+      <c r="S47" t="n">
+        <v>226</v>
+      </c>
+      <c r="T47" t="n">
+        <v>43</v>
+      </c>
+      <c r="U47" t="n">
+        <v>219</v>
+      </c>
+      <c r="V47" t="n">
+        <v>93.24030839396242</v>
+      </c>
+      <c r="W47" t="n">
+        <v>81.98052864803893</v>
       </c>
     </row>
     <row r="48">
@@ -3428,7 +4632,31 @@
         <v>4.720581643413406</v>
       </c>
       <c r="O48" t="n">
+        <v>222</v>
+      </c>
+      <c r="P48" t="n">
+        <v>305</v>
+      </c>
+      <c r="Q48" t="n">
         <v>0.2854867018479598</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0.9630562561179331</v>
+      </c>
+      <c r="S48" t="n">
+        <v>186</v>
+      </c>
+      <c r="T48" t="n">
+        <v>39</v>
+      </c>
+      <c r="U48" t="n">
+        <v>155</v>
+      </c>
+      <c r="V48" t="n">
+        <v>92.8768418564337</v>
+      </c>
+      <c r="W48" t="n">
+        <v>81.47137677656841</v>
       </c>
     </row>
     <row r="49">
@@ -3485,7 +4713,31 @@
         <v>4.593411381103346</v>
       </c>
       <c r="O49" t="n">
+        <v>184</v>
+      </c>
+      <c r="P49" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q49" t="n">
         <v>0.2932413800296404</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0.9605003139816221</v>
+      </c>
+      <c r="S49" t="n">
+        <v>156</v>
+      </c>
+      <c r="T49" t="n">
+        <v>30</v>
+      </c>
+      <c r="U49" t="n">
+        <v>161</v>
+      </c>
+      <c r="V49" t="n">
+        <v>93.46125339701887</v>
+      </c>
+      <c r="W49" t="n">
+        <v>79.18843417899508</v>
       </c>
     </row>
     <row r="50">
@@ -3542,7 +4794,31 @@
         <v>4.59032512764368</v>
       </c>
       <c r="O50" t="n">
+        <v>214</v>
+      </c>
+      <c r="P50" t="n">
+        <v>313</v>
+      </c>
+      <c r="Q50" t="n">
         <v>0.2685946379376621</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0.9745480440855695</v>
+      </c>
+      <c r="S50" t="n">
+        <v>176</v>
+      </c>
+      <c r="T50" t="n">
+        <v>41</v>
+      </c>
+      <c r="U50" t="n">
+        <v>169</v>
+      </c>
+      <c r="V50" t="n">
+        <v>92.95592342802642</v>
+      </c>
+      <c r="W50" t="n">
+        <v>81.72562716981393</v>
       </c>
     </row>
     <row r="51">
@@ -3599,7 +4875,31 @@
         <v>5.198376090641221</v>
       </c>
       <c r="O51" t="n">
+        <v>264</v>
+      </c>
+      <c r="P51" t="n">
+        <v>356</v>
+      </c>
+      <c r="Q51" t="n">
         <v>0.2703424787425938</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.8948284501938498</v>
+      </c>
+      <c r="S51" t="n">
+        <v>218</v>
+      </c>
+      <c r="T51" t="n">
+        <v>55</v>
+      </c>
+      <c r="U51" t="n">
+        <v>149</v>
+      </c>
+      <c r="V51" t="n">
+        <v>92.13744903902155</v>
+      </c>
+      <c r="W51" t="n">
+        <v>85.10198095969912</v>
       </c>
     </row>
     <row r="52">
@@ -3656,7 +4956,31 @@
         <v>4.9986268963582</v>
       </c>
       <c r="O52" t="n">
+        <v>191</v>
+      </c>
+      <c r="P52" t="n">
+        <v>254</v>
+      </c>
+      <c r="Q52" t="n">
         <v>0.2627299208379662</v>
+      </c>
+      <c r="R52" t="n">
+        <v>0.8972046342217571</v>
+      </c>
+      <c r="S52" t="n">
+        <v>164</v>
+      </c>
+      <c r="T52" t="n">
+        <v>27</v>
+      </c>
+      <c r="U52" t="n">
+        <v>98</v>
+      </c>
+      <c r="V52" t="n">
+        <v>92.75161588180978</v>
+      </c>
+      <c r="W52" t="n">
+        <v>83.89644687352467</v>
       </c>
     </row>
     <row r="53">
@@ -3713,7 +5037,31 @@
         <v>4.611128413260047</v>
       </c>
       <c r="O53" t="n">
+        <v>134</v>
+      </c>
+      <c r="P53" t="n">
+        <v>160</v>
+      </c>
+      <c r="Q53" t="n">
         <v>0.2658811733944344</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0.8771866846752886</v>
+      </c>
+      <c r="S53" t="n">
+        <v>108</v>
+      </c>
+      <c r="T53" t="n">
+        <v>26</v>
+      </c>
+      <c r="U53" t="n">
+        <v>57</v>
+      </c>
+      <c r="V53" t="n">
+        <v>89.88276858840534</v>
+      </c>
+      <c r="W53" t="n">
+        <v>86.73165111284986</v>
       </c>
     </row>
     <row r="54">
@@ -3770,7 +5118,31 @@
         <v>4.793987812521896</v>
       </c>
       <c r="O54" t="n">
+        <v>215</v>
+      </c>
+      <c r="P54" t="n">
+        <v>311</v>
+      </c>
+      <c r="Q54" t="n">
         <v>0.2893231873169808</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0.9594505910817277</v>
+      </c>
+      <c r="S54" t="n">
+        <v>178</v>
+      </c>
+      <c r="T54" t="n">
+        <v>39</v>
+      </c>
+      <c r="U54" t="n">
+        <v>166</v>
+      </c>
+      <c r="V54" t="n">
+        <v>92.63746505125815</v>
+      </c>
+      <c r="W54" t="n">
+        <v>80.12279968632528</v>
       </c>
     </row>
     <row r="55">
@@ -3827,7 +5199,31 @@
         <v>5.0691574693687</v>
       </c>
       <c r="O55" t="n">
+        <v>202</v>
+      </c>
+      <c r="P55" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q55" t="n">
         <v>0.2485457638204581</v>
+      </c>
+      <c r="R55" t="n">
+        <v>0.9401104258539872</v>
+      </c>
+      <c r="S55" t="n">
+        <v>178</v>
+      </c>
+      <c r="T55" t="n">
+        <v>25</v>
+      </c>
+      <c r="U55" t="n">
+        <v>117</v>
+      </c>
+      <c r="V55" t="n">
+        <v>94.39451048613124</v>
+      </c>
+      <c r="W55" t="n">
+        <v>84.30589048680227</v>
       </c>
     </row>
     <row r="56">
@@ -3884,7 +5280,31 @@
         <v>4.923327216204122</v>
       </c>
       <c r="O56" t="n">
+        <v>184</v>
+      </c>
+      <c r="P56" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q56" t="n">
         <v>0.2283391735577567</v>
+      </c>
+      <c r="R56" t="n">
+        <v>0.9588958952267727</v>
+      </c>
+      <c r="S56" t="n">
+        <v>161</v>
+      </c>
+      <c r="T56" t="n">
+        <v>24</v>
+      </c>
+      <c r="U56" t="n">
+        <v>105</v>
+      </c>
+      <c r="V56" t="n">
+        <v>95.39858552344363</v>
+      </c>
+      <c r="W56" t="n">
+        <v>86.38140217777021</v>
       </c>
     </row>
     <row r="57">
@@ -3941,7 +5361,31 @@
         <v>4.923126530275171</v>
       </c>
       <c r="O57" t="n">
+        <v>184</v>
+      </c>
+      <c r="P57" t="n">
+        <v>246</v>
+      </c>
+      <c r="Q57" t="n">
         <v>0.2589215361035365</v>
+      </c>
+      <c r="R57" t="n">
+        <v>0.8976155117475519</v>
+      </c>
+      <c r="S57" t="n">
+        <v>164</v>
+      </c>
+      <c r="T57" t="n">
+        <v>21</v>
+      </c>
+      <c r="U57" t="n">
+        <v>97</v>
+      </c>
+      <c r="V57" t="n">
+        <v>93.85783298826777</v>
+      </c>
+      <c r="W57" t="n">
+        <v>84.14475802959191</v>
       </c>
     </row>
     <row r="58">
@@ -3998,7 +5442,31 @@
         <v>5.086791409382254</v>
       </c>
       <c r="O58" t="n">
+        <v>203</v>
+      </c>
+      <c r="P58" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q58" t="n">
         <v>0.2572627020835984</v>
+      </c>
+      <c r="R58" t="n">
+        <v>0.8991747792727228</v>
+      </c>
+      <c r="S58" t="n">
+        <v>175</v>
+      </c>
+      <c r="T58" t="n">
+        <v>28</v>
+      </c>
+      <c r="U58" t="n">
+        <v>115</v>
+      </c>
+      <c r="V58" t="n">
+        <v>93.33130328867236</v>
+      </c>
+      <c r="W58" t="n">
+        <v>83.23064073517614</v>
       </c>
     </row>
     <row r="59">
@@ -4055,7 +5523,31 @@
         <v>5.064734769931102</v>
       </c>
       <c r="O59" t="n">
+        <v>230</v>
+      </c>
+      <c r="P59" t="n">
+        <v>299</v>
+      </c>
+      <c r="Q59" t="n">
         <v>0.248845288942957</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0.9250221623055163</v>
+      </c>
+      <c r="S59" t="n">
+        <v>191</v>
+      </c>
+      <c r="T59" t="n">
+        <v>40</v>
+      </c>
+      <c r="U59" t="n">
+        <v>122</v>
+      </c>
+      <c r="V59" t="n">
+        <v>92.42796332678455</v>
+      </c>
+      <c r="W59" t="n">
+        <v>85.75967917111045</v>
       </c>
     </row>
     <row r="60">
@@ -4112,7 +5604,31 @@
         <v>4.487747967477103</v>
       </c>
       <c r="O60" t="n">
+        <v>166</v>
+      </c>
+      <c r="P60" t="n">
+        <v>247</v>
+      </c>
+      <c r="Q60" t="n">
         <v>0.2632830454531033</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0.9730515810992127</v>
+      </c>
+      <c r="S60" t="n">
+        <v>135</v>
+      </c>
+      <c r="T60" t="n">
+        <v>31</v>
+      </c>
+      <c r="U60" t="n">
+        <v>138</v>
+      </c>
+      <c r="V60" t="n">
+        <v>91.06178175031923</v>
+      </c>
+      <c r="W60" t="n">
+        <v>79.99812122423459</v>
       </c>
     </row>
     <row r="61">
@@ -4169,7 +5685,31 @@
         <v>4.449667062449</v>
       </c>
       <c r="O61" t="n">
+        <v>153</v>
+      </c>
+      <c r="P61" t="n">
+        <v>237</v>
+      </c>
+      <c r="Q61" t="n">
         <v>0.2739717276827358</v>
+      </c>
+      <c r="R61" t="n">
+        <v>0.96982868297164</v>
+      </c>
+      <c r="S61" t="n">
+        <v>131</v>
+      </c>
+      <c r="T61" t="n">
+        <v>22</v>
+      </c>
+      <c r="U61" t="n">
+        <v>132</v>
+      </c>
+      <c r="V61" t="n">
+        <v>93.79879054425508</v>
+      </c>
+      <c r="W61" t="n">
+        <v>79.1178961536627</v>
       </c>
     </row>
     <row r="62">
@@ -4226,7 +5766,31 @@
         <v>4.488940656499014</v>
       </c>
       <c r="O62" t="n">
+        <v>167</v>
+      </c>
+      <c r="P62" t="n">
+        <v>236</v>
+      </c>
+      <c r="Q62" t="n">
         <v>0.2737750514559069</v>
+      </c>
+      <c r="R62" t="n">
+        <v>0.9689792019260394</v>
+      </c>
+      <c r="S62" t="n">
+        <v>134</v>
+      </c>
+      <c r="T62" t="n">
+        <v>34</v>
+      </c>
+      <c r="U62" t="n">
+        <v>131</v>
+      </c>
+      <c r="V62" t="n">
+        <v>90.43442790128492</v>
+      </c>
+      <c r="W62" t="n">
+        <v>80.21580456677498</v>
       </c>
     </row>
     <row r="63">
@@ -4283,7 +5847,31 @@
         <v>4.746486831567949</v>
       </c>
       <c r="O63" t="n">
+        <v>213</v>
+      </c>
+      <c r="P63" t="n">
+        <v>303</v>
+      </c>
+      <c r="Q63" t="n">
         <v>0.277801437874216</v>
+      </c>
+      <c r="R63" t="n">
+        <v>0.9656736155926207</v>
+      </c>
+      <c r="S63" t="n">
+        <v>174</v>
+      </c>
+      <c r="T63" t="n">
+        <v>45</v>
+      </c>
+      <c r="U63" t="n">
+        <v>162</v>
+      </c>
+      <c r="V63" t="n">
+        <v>90.86633287816719</v>
+      </c>
+      <c r="W63" t="n">
+        <v>81.77046655982045</v>
       </c>
     </row>
     <row r="64">
@@ -4340,7 +5928,31 @@
         <v>4.358451257105805</v>
       </c>
       <c r="O64" t="n">
+        <v>137</v>
+      </c>
+      <c r="P64" t="n">
+        <v>184</v>
+      </c>
+      <c r="Q64" t="n">
         <v>0.2686948952785486</v>
+      </c>
+      <c r="R64" t="n">
+        <v>0.9601508395037023</v>
+      </c>
+      <c r="S64" t="n">
+        <v>115</v>
+      </c>
+      <c r="T64" t="n">
+        <v>22</v>
+      </c>
+      <c r="U64" t="n">
+        <v>93</v>
+      </c>
+      <c r="V64" t="n">
+        <v>92.63436368699527</v>
+      </c>
+      <c r="W64" t="n">
+        <v>82.26854694354549</v>
       </c>
     </row>
     <row r="65">
@@ -4397,7 +6009,31 @@
         <v>4.296682138811668</v>
       </c>
       <c r="O65" t="n">
+        <v>113</v>
+      </c>
+      <c r="P65" t="n">
+        <v>162</v>
+      </c>
+      <c r="Q65" t="n">
         <v>0.2804191380788239</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0.9473335164120311</v>
+      </c>
+      <c r="S65" t="n">
+        <v>97</v>
+      </c>
+      <c r="T65" t="n">
+        <v>16</v>
+      </c>
+      <c r="U65" t="n">
+        <v>86</v>
+      </c>
+      <c r="V65" t="n">
+        <v>91.56584860006916</v>
+      </c>
+      <c r="W65" t="n">
+        <v>79.27194273055848</v>
       </c>
     </row>
     <row r="66">
@@ -4454,7 +6090,31 @@
         <v>4.538688438407363</v>
       </c>
       <c r="O66" t="n">
+        <v>193</v>
+      </c>
+      <c r="P66" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q66" t="n">
         <v>0.2700918684599101</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0.9707614809182677</v>
+      </c>
+      <c r="S66" t="n">
+        <v>154</v>
+      </c>
+      <c r="T66" t="n">
+        <v>39</v>
+      </c>
+      <c r="U66" t="n">
+        <v>129</v>
+      </c>
+      <c r="V66" t="n">
+        <v>91.06605277138304</v>
+      </c>
+      <c r="W66" t="n">
+        <v>82.62788141211865</v>
       </c>
     </row>
     <row r="67">
@@ -4511,7 +6171,31 @@
         <v>4.685229933478695</v>
       </c>
       <c r="O67" t="n">
+        <v>190</v>
+      </c>
+      <c r="P67" t="n">
+        <v>292</v>
+      </c>
+      <c r="Q67" t="n">
         <v>0.2747961933184368</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0.9688528230007389</v>
+      </c>
+      <c r="S67" t="n">
+        <v>161</v>
+      </c>
+      <c r="T67" t="n">
+        <v>31</v>
+      </c>
+      <c r="U67" t="n">
+        <v>160</v>
+      </c>
+      <c r="V67" t="n">
+        <v>92.10713018800993</v>
+      </c>
+      <c r="W67" t="n">
+        <v>79.83165135615687</v>
       </c>
     </row>
     <row r="68">
@@ -4568,7 +6252,31 @@
         <v>4.127867245780121</v>
       </c>
       <c r="O68" t="n">
+        <v>107</v>
+      </c>
+      <c r="P68" t="n">
+        <v>151</v>
+      </c>
+      <c r="Q68" t="n">
         <v>0.2690891615576508</v>
+      </c>
+      <c r="R68" t="n">
+        <v>0.9639553290940605</v>
+      </c>
+      <c r="S68" t="n">
+        <v>85</v>
+      </c>
+      <c r="T68" t="n">
+        <v>23</v>
+      </c>
+      <c r="U68" t="n">
+        <v>82</v>
+      </c>
+      <c r="V68" t="n">
+        <v>89.44689514760775</v>
+      </c>
+      <c r="W68" t="n">
+        <v>80.56254910096159</v>
       </c>
     </row>
     <row r="69">
@@ -4625,7 +6333,31 @@
         <v>5.040834697632513</v>
       </c>
       <c r="O69" t="n">
+        <v>220</v>
+      </c>
+      <c r="P69" t="n">
+        <v>287</v>
+      </c>
+      <c r="Q69" t="n">
         <v>0.2739443868143195</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0.8870656626606725</v>
+      </c>
+      <c r="S69" t="n">
+        <v>181</v>
+      </c>
+      <c r="T69" t="n">
+        <v>42</v>
+      </c>
+      <c r="U69" t="n">
+        <v>115</v>
+      </c>
+      <c r="V69" t="n">
+        <v>91.85047987876746</v>
+      </c>
+      <c r="W69" t="n">
+        <v>85.15277608643756</v>
       </c>
     </row>
     <row r="70">
@@ -4682,7 +6414,31 @@
         <v>5.346065192991746</v>
       </c>
       <c r="O70" t="n">
+        <v>288</v>
+      </c>
+      <c r="P70" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q70" t="n">
         <v>0.2675543077298151</v>
+      </c>
+      <c r="R70" t="n">
+        <v>0.9135920628935402</v>
+      </c>
+      <c r="S70" t="n">
+        <v>241</v>
+      </c>
+      <c r="T70" t="n">
+        <v>54</v>
+      </c>
+      <c r="U70" t="n">
+        <v>171</v>
+      </c>
+      <c r="V70" t="n">
+        <v>92.61955566712689</v>
+      </c>
+      <c r="W70" t="n">
+        <v>83.28884876457812</v>
       </c>
     </row>
     <row r="71">
@@ -4739,7 +6495,31 @@
         <v>5.314311848432592</v>
       </c>
       <c r="O71" t="n">
+        <v>300</v>
+      </c>
+      <c r="P71" t="n">
+        <v>401</v>
+      </c>
+      <c r="Q71" t="n">
         <v>0.2650126215301735</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0.9181501987985393</v>
+      </c>
+      <c r="S71" t="n">
+        <v>256</v>
+      </c>
+      <c r="T71" t="n">
+        <v>52</v>
+      </c>
+      <c r="U71" t="n">
+        <v>170</v>
+      </c>
+      <c r="V71" t="n">
+        <v>93.43375596138188</v>
+      </c>
+      <c r="W71" t="n">
+        <v>84.20531356204233</v>
       </c>
     </row>
     <row r="72">
@@ -4796,7 +6576,31 @@
         <v>4.938517906954239</v>
       </c>
       <c r="O72" t="n">
+        <v>183</v>
+      </c>
+      <c r="P72" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q72" t="n">
         <v>0.2719827874058284</v>
+      </c>
+      <c r="R72" t="n">
+        <v>0.8993897970415016</v>
+      </c>
+      <c r="S72" t="n">
+        <v>147</v>
+      </c>
+      <c r="T72" t="n">
+        <v>36</v>
+      </c>
+      <c r="U72" t="n">
+        <v>108</v>
+      </c>
+      <c r="V72" t="n">
+        <v>90.22061244649325</v>
+      </c>
+      <c r="W72" t="n">
+        <v>80.97803368039793</v>
       </c>
     </row>
     <row r="73">
@@ -4853,7 +6657,31 @@
         <v>5.201809091677285</v>
       </c>
       <c r="O73" t="n">
+        <v>258</v>
+      </c>
+      <c r="P73" t="n">
+        <v>327</v>
+      </c>
+      <c r="Q73" t="n">
         <v>0.2605053878028613</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0.9209381511658592</v>
+      </c>
+      <c r="S73" t="n">
+        <v>208</v>
+      </c>
+      <c r="T73" t="n">
+        <v>52</v>
+      </c>
+      <c r="U73" t="n">
+        <v>136</v>
+      </c>
+      <c r="V73" t="n">
+        <v>90.23208734003325</v>
+      </c>
+      <c r="W73" t="n">
+        <v>83.684944405057</v>
       </c>
     </row>
     <row r="74">
@@ -4910,7 +6738,31 @@
         <v>5.07582422587299</v>
       </c>
       <c r="O74" t="n">
+        <v>211</v>
+      </c>
+      <c r="P74" t="n">
+        <v>267</v>
+      </c>
+      <c r="Q74" t="n">
         <v>0.2931282330939343</v>
+      </c>
+      <c r="R74" t="n">
+        <v>0.8541186990102084</v>
+      </c>
+      <c r="S74" t="n">
+        <v>165</v>
+      </c>
+      <c r="T74" t="n">
+        <v>47</v>
+      </c>
+      <c r="U74" t="n">
+        <v>112</v>
+      </c>
+      <c r="V74" t="n">
+        <v>88.49303849303848</v>
+      </c>
+      <c r="W74" t="n">
+        <v>81.44617402807934</v>
       </c>
     </row>
     <row r="75">
@@ -4967,7 +6819,31 @@
         <v>4.948808225371879</v>
       </c>
       <c r="O75" t="n">
+        <v>174</v>
+      </c>
+      <c r="P75" t="n">
+        <v>240</v>
+      </c>
+      <c r="Q75" t="n">
         <v>0.2710088589395877</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0.8956318865298839</v>
+      </c>
+      <c r="S75" t="n">
+        <v>148</v>
+      </c>
+      <c r="T75" t="n">
+        <v>26</v>
+      </c>
+      <c r="U75" t="n">
+        <v>99</v>
+      </c>
+      <c r="V75" t="n">
+        <v>93.17724068479356</v>
+      </c>
+      <c r="W75" t="n">
+        <v>81.46992713386648</v>
       </c>
     </row>
     <row r="76">
@@ -5024,7 +6900,31 @@
         <v>4.037207334187973</v>
       </c>
       <c r="O76" t="n">
+        <v>83</v>
+      </c>
+      <c r="P76" t="n">
+        <v>135</v>
+      </c>
+      <c r="Q76" t="n">
         <v>0.3066380611163251</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0.9468108462536275</v>
+      </c>
+      <c r="S76" t="n">
+        <v>67</v>
+      </c>
+      <c r="T76" t="n">
+        <v>16</v>
+      </c>
+      <c r="U76" t="n">
+        <v>87</v>
+      </c>
+      <c r="V76" t="n">
+        <v>90.58277878604557</v>
+      </c>
+      <c r="W76" t="n">
+        <v>77.15612620444328</v>
       </c>
     </row>
     <row r="77">
@@ -5081,7 +6981,31 @@
         <v>5.24373219381151</v>
       </c>
       <c r="O77" t="n">
+        <v>310</v>
+      </c>
+      <c r="P77" t="n">
+        <v>429</v>
+      </c>
+      <c r="Q77" t="n">
         <v>0.2567669657322042</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0.9214280977944701</v>
+      </c>
+      <c r="S77" t="n">
+        <v>260</v>
+      </c>
+      <c r="T77" t="n">
+        <v>60</v>
+      </c>
+      <c r="U77" t="n">
+        <v>180</v>
+      </c>
+      <c r="V77" t="n">
+        <v>92.84466065271808</v>
+      </c>
+      <c r="W77" t="n">
+        <v>85.96246292943522</v>
       </c>
     </row>
     <row r="78">
@@ -5138,7 +7062,31 @@
         <v>4.642928809886867</v>
       </c>
       <c r="O78" t="n">
+        <v>229</v>
+      </c>
+      <c r="P78" t="n">
+        <v>327</v>
+      </c>
+      <c r="Q78" t="n">
         <v>0.2619752694225917</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0.9773297885033696</v>
+      </c>
+      <c r="S78" t="n">
+        <v>190</v>
+      </c>
+      <c r="T78" t="n">
+        <v>40</v>
+      </c>
+      <c r="U78" t="n">
+        <v>166</v>
+      </c>
+      <c r="V78" t="n">
+        <v>92.95654457135355</v>
+      </c>
+      <c r="W78" t="n">
+        <v>82.54394333188971</v>
       </c>
     </row>
     <row r="79">
@@ -5195,7 +7143,31 @@
         <v>5.101958906237616</v>
       </c>
       <c r="O79" t="n">
+        <v>265</v>
+      </c>
+      <c r="P79" t="n">
+        <v>368</v>
+      </c>
+      <c r="Q79" t="n">
         <v>0.2411020763865226</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0.9363180521840262</v>
+      </c>
+      <c r="S79" t="n">
+        <v>237</v>
+      </c>
+      <c r="T79" t="n">
+        <v>35</v>
+      </c>
+      <c r="U79" t="n">
+        <v>144</v>
+      </c>
+      <c r="V79" t="n">
+        <v>95.13447290123096</v>
+      </c>
+      <c r="W79" t="n">
+        <v>86.53706701396928</v>
       </c>
     </row>
     <row r="80">
@@ -5252,7 +7224,31 @@
         <v>4.938340692114959</v>
       </c>
       <c r="O80" t="n">
+        <v>221</v>
+      </c>
+      <c r="P80" t="n">
+        <v>287</v>
+      </c>
+      <c r="Q80" t="n">
         <v>0.2368423677303973</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0.9192076451104011</v>
+      </c>
+      <c r="S80" t="n">
+        <v>195</v>
+      </c>
+      <c r="T80" t="n">
+        <v>27</v>
+      </c>
+      <c r="U80" t="n">
+        <v>110</v>
+      </c>
+      <c r="V80" t="n">
+        <v>95.71165296285795</v>
+      </c>
+      <c r="W80" t="n">
+        <v>87.85469223959099</v>
       </c>
     </row>
     <row r="81">
@@ -5309,7 +7305,31 @@
         <v>4.825142406965177</v>
       </c>
       <c r="O81" t="n">
+        <v>172</v>
+      </c>
+      <c r="P81" t="n">
+        <v>224</v>
+      </c>
+      <c r="Q81" t="n">
         <v>0.2399069609089002</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0.900801799049412</v>
+      </c>
+      <c r="S81" t="n">
+        <v>147</v>
+      </c>
+      <c r="T81" t="n">
+        <v>25</v>
+      </c>
+      <c r="U81" t="n">
+        <v>81</v>
+      </c>
+      <c r="V81" t="n">
+        <v>93.60269360269359</v>
+      </c>
+      <c r="W81" t="n">
+        <v>85.49609083883678</v>
       </c>
     </row>
     <row r="82">
@@ -5366,7 +7386,31 @@
         <v>4.584442138079433</v>
       </c>
       <c r="O82" t="n">
+        <v>183</v>
+      </c>
+      <c r="P82" t="n">
+        <v>252</v>
+      </c>
+      <c r="Q82" t="n">
         <v>0.2757342033756477</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0.965872350727799</v>
+      </c>
+      <c r="S82" t="n">
+        <v>150</v>
+      </c>
+      <c r="T82" t="n">
+        <v>34</v>
+      </c>
+      <c r="U82" t="n">
+        <v>132</v>
+      </c>
+      <c r="V82" t="n">
+        <v>90.82531230800737</v>
+      </c>
+      <c r="W82" t="n">
+        <v>80.35239323847694</v>
       </c>
     </row>
     <row r="83">
@@ -5423,7 +7467,31 @@
         <v>4.427288386355573</v>
       </c>
       <c r="O83" t="n">
+        <v>154</v>
+      </c>
+      <c r="P83" t="n">
+        <v>237</v>
+      </c>
+      <c r="Q83" t="n">
         <v>0.280630853306521</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0.9691524034797644</v>
+      </c>
+      <c r="S83" t="n">
+        <v>125</v>
+      </c>
+      <c r="T83" t="n">
+        <v>29</v>
+      </c>
+      <c r="U83" t="n">
+        <v>140</v>
+      </c>
+      <c r="V83" t="n">
+        <v>91.80834621329213</v>
+      </c>
+      <c r="W83" t="n">
+        <v>79.3815636287263</v>
       </c>
     </row>
     <row r="84">
@@ -5480,7 +7548,31 @@
         <v>4.258351426467049</v>
       </c>
       <c r="O84" t="n">
+        <v>141</v>
+      </c>
+      <c r="P84" t="n">
+        <v>205</v>
+      </c>
+      <c r="Q84" t="n">
         <v>0.27940027743208</v>
+      </c>
+      <c r="R84" t="n">
+        <v>0.9724175941197054</v>
+      </c>
+      <c r="S84" t="n">
+        <v>113</v>
+      </c>
+      <c r="T84" t="n">
+        <v>28</v>
+      </c>
+      <c r="U84" t="n">
+        <v>119</v>
+      </c>
+      <c r="V84" t="n">
+        <v>91.85136178189435</v>
+      </c>
+      <c r="W84" t="n">
+        <v>80.41692164082933</v>
       </c>
     </row>
     <row r="85">
@@ -5537,7 +7629,31 @@
         <v>4.700748223279477</v>
       </c>
       <c r="O85" t="n">
+        <v>164</v>
+      </c>
+      <c r="P85" t="n">
+        <v>236</v>
+      </c>
+      <c r="Q85" t="n">
         <v>0.2503889858940836</v>
+      </c>
+      <c r="R85" t="n">
+        <v>0.9158650183797254</v>
+      </c>
+      <c r="S85" t="n">
+        <v>153</v>
+      </c>
+      <c r="T85" t="n">
+        <v>20</v>
+      </c>
+      <c r="U85" t="n">
+        <v>100</v>
+      </c>
+      <c r="V85" t="n">
+        <v>96.38639794015805</v>
+      </c>
+      <c r="W85" t="n">
+        <v>83.35125782445725</v>
       </c>
     </row>
     <row r="86">
@@ -5594,7 +7710,31 @@
         <v>4.307786660775069</v>
       </c>
       <c r="O86" t="n">
+        <v>150</v>
+      </c>
+      <c r="P86" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q86" t="n">
         <v>0.227968590149114</v>
+      </c>
+      <c r="R86" t="n">
+        <v>0.9630353129447141</v>
+      </c>
+      <c r="S86" t="n">
+        <v>136</v>
+      </c>
+      <c r="T86" t="n">
+        <v>15</v>
+      </c>
+      <c r="U86" t="n">
+        <v>99</v>
+      </c>
+      <c r="V86" t="n">
+        <v>97.64246565057437</v>
+      </c>
+      <c r="W86" t="n">
+        <v>86.70524895060433</v>
       </c>
     </row>
     <row r="87">
@@ -5651,7 +7791,31 @@
         <v>4.796694279400795</v>
       </c>
       <c r="O87" t="n">
+        <v>265</v>
+      </c>
+      <c r="P87" t="n">
+        <v>385</v>
+      </c>
+      <c r="Q87" t="n">
         <v>0.2759835837192705</v>
+      </c>
+      <c r="R87" t="n">
+        <v>0.9763215311901919</v>
+      </c>
+      <c r="S87" t="n">
+        <v>214</v>
+      </c>
+      <c r="T87" t="n">
+        <v>56</v>
+      </c>
+      <c r="U87" t="n">
+        <v>207</v>
+      </c>
+      <c r="V87" t="n">
+        <v>91.89740287615368</v>
+      </c>
+      <c r="W87" t="n">
+        <v>81.7152636674175</v>
       </c>
     </row>
     <row r="88">
@@ -5708,7 +7872,31 @@
         <v>4.742177999043804</v>
       </c>
       <c r="O88" t="n">
+        <v>181</v>
+      </c>
+      <c r="P88" t="n">
+        <v>276</v>
+      </c>
+      <c r="Q88" t="n">
         <v>0.2425458882024158</v>
+      </c>
+      <c r="R88" t="n">
+        <v>0.938519572845514</v>
+      </c>
+      <c r="S88" t="n">
+        <v>167</v>
+      </c>
+      <c r="T88" t="n">
+        <v>22</v>
+      </c>
+      <c r="U88" t="n">
+        <v>112</v>
+      </c>
+      <c r="V88" t="n">
+        <v>96.54934437543135</v>
+      </c>
+      <c r="W88" t="n">
+        <v>86.90580142788363</v>
       </c>
     </row>
   </sheetData>
@@ -5717,6 +7905,212 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="33" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="37" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="33" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tipo de muestra</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Bray-Curtis misma muestra (media)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Bray-Curtis misma muestra (desv. est.)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Pearson misma muestra (media)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Pearson misma muestra (desv. est.)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Especies compartidas (media)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Especies compartidas (desv. est.)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Shannon (este trabajo) (media)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Shannon (este trabajo) (desv. est.)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Shannon (artículo) (media)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Shannon (artículo) (desv. est.)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Riqueza (este trabajo) (media)</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Riqueza (este trabajo) (desv. est.)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Riqueza (artículo) (media)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Riqueza (artículo) (desv. est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bolsa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F2" t="n">
+        <v>190.487</v>
+      </c>
+      <c r="G2" t="n">
+        <v>38.999</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.763</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="J2" t="n">
+        <v>4.981</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="L2" t="n">
+        <v>217.821</v>
+      </c>
+      <c r="M2" t="n">
+        <v>45.633</v>
+      </c>
+      <c r="N2" t="n">
+        <v>301.718</v>
+      </c>
+      <c r="O2" t="n">
+        <v>62.365</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Suelo</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="F3" t="n">
+        <v>157.771</v>
+      </c>
+      <c r="G3" t="n">
+        <v>45.655</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.372</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4.579</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L3" t="n">
+        <v>188.292</v>
+      </c>
+      <c r="M3" t="n">
+        <v>52.494</v>
+      </c>
+      <c r="N3" t="n">
+        <v>276.958</v>
+      </c>
+      <c r="O3" t="n">
+        <v>76.553</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>